<commit_message>
feat: wire 3-reference Gemini image generation pipeline and configure Row 184
</commit_message>
<xml_diff>
--- a/Vinayak’s Copy of Zara Khan.xlsx
+++ b/Vinayak’s Copy of Zara Khan.xlsx
@@ -8256,7 +8256,7 @@
       <c r="G184" s="27" t="inlineStr"/>
       <c r="H184" s="27" t="inlineStr">
         <is>
-          <t>https://in.pinterest.com/pin/1105985746020500854/</t>
+          <t>https://images.unsplash.com/photo-1554118811-1e0d58224f24?auto=format&amp;fit=crop&amp;w=1080&amp;q=80</t>
         </is>
       </c>
       <c r="I184" s="27" t="inlineStr">
@@ -8266,12 +8266,12 @@
       </c>
       <c r="J184" s="27" t="inlineStr">
         <is>
-          <t>ZARA_KHAN.png</t>
+          <t>https://images.unsplash.com/photo-1583391733956-3750e0ff4e8b?auto=format&amp;fit=crop&amp;w=1080&amp;q=80</t>
         </is>
       </c>
       <c r="K184" s="27" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>prompted</t>
         </is>
       </c>
       <c r="L184" s="27" t="inlineStr">
@@ -8281,7 +8281,15 @@
       </c>
       <c r="M184" s="27" t="inlineStr"/>
       <c r="N184" s="27" t="inlineStr"/>
-      <c r="O184" s="27" t="inlineStr"/>
+      <c r="O184" s="27" t="inlineStr">
+        <is>
+          <t>[Post · photo · 9:16 · 1152x2048 · Gemini 3.1 Flash Lite Image / Nano Banana]
+Cinematic 35mm film photography of Zara Khan in a quiet sunlit South Mumbai heritage cafe patio. She has long dark natural wavy hair, expressive warm brown eyes, and a relaxed candid smile. She is wearing an ivory linen button-up shirt and layered delicate gold necklaces, holding a coffee cup and reading a book. Natural warm morning light streams through vintage wooden blinds casting soft shadows. Photorealistic textures, soft depth of field, authentic candid lifestyle influencer aesthetic, Fujifilm color grade.
+Wardrobe &amp; Styling: Ivory linen button-up shirt, delicate layered gold necklaces, authentic Lucknow craftsmanship.
+Setting &amp; Environment: South Mumbai colonial heritage cafe patio with vintage wooden blinds and morning sun.
+Avoid: plastic skin, artificial lighting, CGI, 3D render, modern minimalist sterile aesthetic, heavy makeup, distorted anatomy, blurry, oversaturated colors.</t>
+        </is>
+      </c>
       <c r="P184" s="27" t="n"/>
       <c r="Q184" s="27" t="n"/>
       <c r="R184" s="27" t="n"/>

</xml_diff>

<commit_message>
feat: document multimodal pipeline progress, update README, and package Day 101-103 assets
</commit_message>
<xml_diff>
--- a/Vinayak’s Copy of Zara Khan.xlsx
+++ b/Vinayak’s Copy of Zara Khan.xlsx
@@ -8304,21 +8304,65 @@
       <c r="AA184" s="27" t="n"/>
     </row>
     <row r="185">
-      <c r="A185" s="27" t="n"/>
-      <c r="B185" s="27" t="n"/>
-      <c r="C185" s="27" t="n"/>
-      <c r="D185" s="27" t="n"/>
-      <c r="E185" s="27" t="n"/>
-      <c r="F185" s="27" t="n"/>
-      <c r="G185" s="27" t="n"/>
-      <c r="H185" s="27" t="n"/>
-      <c r="I185" s="27" t="n"/>
-      <c r="J185" s="27" t="n"/>
-      <c r="K185" s="27" t="n"/>
-      <c r="L185" s="27" t="n"/>
-      <c r="M185" s="27" t="n"/>
-      <c r="N185" s="27" t="n"/>
-      <c r="O185" s="27" t="n"/>
+      <c r="A185" s="27" t="inlineStr">
+        <is>
+          <t>Test Day 102</t>
+        </is>
+      </c>
+      <c r="B185" s="27" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="C185" s="27" t="inlineStr">
+        <is>
+          <t>Zara Khan quiet luxury evening aesthetic in modern Fort art gallery admiring contemporary paintings</t>
+        </is>
+      </c>
+      <c r="D185" s="27" t="inlineStr">
+        <is>
+          <t>Modern art gallery white walls with framed artworks and reflective polished floors, deep royal purple silk saree with intricate gold zari border, sleeveless black velvet blouse, gold jhumkas, serene poise, Zara Khan face lock consistency</t>
+        </is>
+      </c>
+      <c r="E185" s="27" t="inlineStr">
+        <is>
+          <t>Contemporary ambient gallery cello and acoustic strings</t>
+        </is>
+      </c>
+      <c r="F185" s="27" t="inlineStr">
+        <is>
+          <t>Art speaks loudest in the quiet spaces between galleries. An evening surrounded by perspective in Fort.</t>
+        </is>
+      </c>
+      <c r="G185" s="27" t="inlineStr"/>
+      <c r="H185" s="27" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1518998053901-5348d3961a04?auto=format&amp;fit=crop&amp;w=1080&amp;q=80</t>
+        </is>
+      </c>
+      <c r="I185" s="27" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1IaeGtZF6cLdXTyREF6HiDwyY3x9_0sOf</t>
+        </is>
+      </c>
+      <c r="J185" s="27" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1610030469983-98e550d6193c?auto=format&amp;fit=crop&amp;w=1080&amp;q=80</t>
+        </is>
+      </c>
+      <c r="K185" s="27" t="inlineStr">
+        <is>
+          <t>prompted</t>
+        </is>
+      </c>
+      <c r="L185" s="27" t="inlineStr">
+        <is>
+          <t>102</t>
+        </is>
+      </c>
+      <c r="M185" s="27" t="inlineStr"/>
+      <c r="N185" s="27" t="inlineStr"/>
+      <c r="O185" s="27" t="inlineStr"/>
       <c r="P185" s="27" t="n"/>
       <c r="Q185" s="27" t="n"/>
       <c r="R185" s="27" t="n"/>
@@ -8333,21 +8377,65 @@
       <c r="AA185" s="27" t="n"/>
     </row>
     <row r="186">
-      <c r="A186" s="27" t="n"/>
-      <c r="B186" s="27" t="n"/>
-      <c r="C186" s="27" t="n"/>
-      <c r="D186" s="27" t="n"/>
-      <c r="E186" s="27" t="n"/>
-      <c r="F186" s="27" t="n"/>
-      <c r="G186" s="27" t="n"/>
-      <c r="H186" s="27" t="n"/>
-      <c r="I186" s="27" t="n"/>
-      <c r="J186" s="27" t="n"/>
-      <c r="K186" s="27" t="n"/>
-      <c r="L186" s="27" t="n"/>
-      <c r="M186" s="27" t="n"/>
-      <c r="N186" s="27" t="n"/>
-      <c r="O186" s="27" t="n"/>
+      <c r="A186" s="27" t="inlineStr">
+        <is>
+          <t>Test Day 103</t>
+        </is>
+      </c>
+      <c r="B186" s="27" t="inlineStr">
+        <is>
+          <t>Post</t>
+        </is>
+      </c>
+      <c r="C186" s="27" t="inlineStr">
+        <is>
+          <t>Zara Khan heritage library study aesthetic in warm mahogany lounge with antique bookshelves and soft lamp glow</t>
+        </is>
+      </c>
+      <c r="D186" s="27" t="inlineStr">
+        <is>
+          <t>Rich mahogany wood-paneled study with warm pleated lampshades and antique books, vibrant crimson rose and gold Kanjeevaram silk saree with bold zari borders, traditional gold temple jewelry, serene poised smile, Zara Khan face lock consistency</t>
+        </is>
+      </c>
+      <c r="E186" s="27" t="inlineStr">
+        <is>
+          <t>Traditional sitar and warm classical Indian acoustic melody</t>
+        </is>
+      </c>
+      <c r="F186" s="27" t="inlineStr">
+        <is>
+          <t>Surrounded by centuries of stories in the quiet heart of Bombay. Crimson silks and warm lamplight.</t>
+        </is>
+      </c>
+      <c r="G186" s="27" t="inlineStr"/>
+      <c r="H186" s="27" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1590381105924-c72589b9ef3f?auto=format&amp;fit=crop&amp;w=1080&amp;q=80</t>
+        </is>
+      </c>
+      <c r="I186" s="27" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/drive/folders/1IaeGtZF6cLdXTyREF6HiDwyY3x9_0sOf</t>
+        </is>
+      </c>
+      <c r="J186" s="27" t="inlineStr">
+        <is>
+          <t>https://images.unsplash.com/photo-1617627143750-d86bc21e42bb?auto=format&amp;fit=crop&amp;w=1080&amp;q=80</t>
+        </is>
+      </c>
+      <c r="K186" s="27" t="inlineStr">
+        <is>
+          <t>prompted</t>
+        </is>
+      </c>
+      <c r="L186" s="27" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
+      <c r="M186" s="27" t="inlineStr"/>
+      <c r="N186" s="27" t="inlineStr"/>
+      <c r="O186" s="27" t="inlineStr"/>
       <c r="P186" s="27" t="n"/>
       <c r="Q186" s="27" t="n"/>
       <c r="R186" s="27" t="n"/>

</xml_diff>